<commit_message>
Normalize FDI workbook tables
</commit_message>
<xml_diff>
--- a/templates/FDI_Master.xlsx
+++ b/templates/FDI_Master.xlsx
@@ -17,6 +17,7 @@
     <sheet name="MEZ_S01_Form" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="CFL_S01_Form" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="MZL_S01_Form" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FDI_Table_Config" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -285,543 +286,730 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tbl009" displayName="tbl009" ref="A79:B83" headerRowCount="1">
-  <autoFilter ref="A79:B83"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblTarimas_DIN" displayName="tblTarimas_DIN" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tbl010" displayName="tbl010" ref="A95:B98" headerRowCount="1">
-  <autoFilter ref="A95:B98"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblProductos_DIN" displayName="tblProductos_DIN" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl011" displayName="tbl011" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblElementosSeguridad_DIN" displayName="tblElementosSeguridad_DIN" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tbl012" displayName="tbl012" ref="A60:C64" headerRowCount="1">
-  <autoFilter ref="A60:C64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPiezasEspeciales_DIN" displayName="tblPiezasEspeciales_DIN" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tbl013" displayName="tbl013" ref="A67:C70" headerRowCount="1">
-  <autoFilter ref="A67:C70"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblColores_DIN" displayName="tblColores_DIN" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tbl014" displayName="tbl014" ref="A79:B83" headerRowCount="1">
-  <autoFilter ref="A79:B83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblProveedoresExternos_DIN" displayName="tblProveedoresExternos_DIN" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tbl015" displayName="tbl015" ref="A95:B98" headerRowCount="1">
-  <autoFilter ref="A95:B98"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblPiezas_PBK" displayName="tblPiezas_PBK" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tbl016" displayName="tbl016" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblTarimas_PBK" displayName="tblTarimas_PBK" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tbl017" displayName="tbl017" ref="A62:C66" headerRowCount="1">
-  <autoFilter ref="A62:C66"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblProductos_PBK" displayName="tblProductos_PBK" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tbl018" displayName="tbl018" ref="A69:C72" headerRowCount="1">
-  <autoFilter ref="A69:C72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblElementosSeguridad_PBK" displayName="tblElementosSeguridad_PBK" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl001" displayName="tbl001" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblPiezas_SEL" displayName="tblPiezas_SEL" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tbl019" displayName="tbl019" ref="A81:B85" headerRowCount="1">
-  <autoFilter ref="A81:B85"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tblPiezasEspeciales_PBK" displayName="tblPiezasEspeciales_PBK" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tbl020" displayName="tbl020" ref="A97:B100" headerRowCount="1">
-  <autoFilter ref="A97:B100"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tblColores_PBK" displayName="tblColores_PBK" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tbl021" displayName="tbl021" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tblProveedoresExternos_PBK" displayName="tblProveedoresExternos_PBK" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="tbl022" displayName="tbl022" ref="A51:C55" headerRowCount="1">
-  <autoFilter ref="A51:C55"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="tblPiezas_DRV" displayName="tblPiezas_DRV" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tbl023" displayName="tbl023" ref="A58:C61" headerRowCount="1">
-  <autoFilter ref="A58:C61"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tblTarimas_DRV" displayName="tblTarimas_DRV" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tbl024" displayName="tbl024" ref="A70:B74" headerRowCount="1">
-  <autoFilter ref="A70:B74"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tblProductos_DRV" displayName="tblProductos_DRV" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tbl025" displayName="tbl025" ref="A86:B89" headerRowCount="1">
-  <autoFilter ref="A86:B89"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tblElementosSeguridad_DRV" displayName="tblElementosSeguridad_DRV" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tbl026" displayName="tbl026" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tblPiezasEspeciales_DRV" displayName="tblPiezasEspeciales_DRV" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tbl027" displayName="tbl027" ref="A30:F36" headerRowCount="1">
-  <autoFilter ref="A30:F36"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Tipo de producto"/>
-    <tableColumn id="2" name="Largo"/>
-    <tableColumn id="3" name="Ancho"/>
-    <tableColumn id="4" name="Alto"/>
-    <tableColumn id="5" name="Peso/pieza"/>
-    <tableColumn id="6" name="Cant./nivel"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tblColores_DRV" displayName="tblColores_DRV" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tbl028" displayName="tbl028" ref="A63:C67" headerRowCount="1">
-  <autoFilter ref="A63:C67"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tblProveedoresExternos_DRV" displayName="tblProveedoresExternos_DRV" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl002" displayName="tbl002" ref="A52:C56" headerRowCount="1">
-  <autoFilter ref="A52:C56"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblTarimas_SEL" displayName="tblTarimas_SEL" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="tbl029" displayName="tbl029" ref="A70:C73" headerRowCount="1">
-  <autoFilter ref="A70:C73"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="tblPiezas_CAN" displayName="tblPiezas_CAN" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tbl030" displayName="tbl030" ref="A82:B86" headerRowCount="1">
-  <autoFilter ref="A82:B86"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tblTarimas_CAN" displayName="tblTarimas_CAN" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="tbl031" displayName="tbl031" ref="A98:B101" headerRowCount="1">
-  <autoFilter ref="A98:B101"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="tblProductos_CAN" displayName="tblProductos_CAN" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="tbl032" displayName="tbl032" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="tblElementosSeguridad_CAN" displayName="tblElementosSeguridad_CAN" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="tbl033" displayName="tbl033" ref="A30:F36" headerRowCount="1">
-  <autoFilter ref="A30:F36"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Tipo de producto"/>
-    <tableColumn id="2" name="Largo"/>
-    <tableColumn id="3" name="Ancho"/>
-    <tableColumn id="4" name="Alto"/>
-    <tableColumn id="5" name="Peso/pieza"/>
-    <tableColumn id="6" name="Cant./nivel"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="tblPiezasEspeciales_CAN" displayName="tblPiezasEspeciales_CAN" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="tbl034" displayName="tbl034" ref="A56:C60" headerRowCount="1">
-  <autoFilter ref="A56:C60"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="tblColores_CAN" displayName="tblColores_CAN" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="tbl035" displayName="tbl035" ref="A63:C66" headerRowCount="1">
-  <autoFilter ref="A63:C66"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="tblProveedoresExternos_CAN" displayName="tblProveedoresExternos_CAN" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="tbl036" displayName="tbl036" ref="A75:B79" headerRowCount="1">
-  <autoFilter ref="A75:B79"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="tblPiezas_MEZ" displayName="tblPiezas_MEZ" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="tbl037" displayName="tbl037" ref="A91:B94" headerRowCount="1">
-  <autoFilter ref="A91:B94"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="tblTarimas_MEZ" displayName="tblTarimas_MEZ" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="tbl038" displayName="tbl038" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="tblProductos_MEZ" displayName="tblProductos_MEZ" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl003" displayName="tbl003" ref="A59:C62" headerRowCount="1">
-  <autoFilter ref="A59:C62"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblProductos_SEL" displayName="tblProductos_SEL" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="tbl039" displayName="tbl039" ref="A49:F53" headerRowCount="1">
-  <autoFilter ref="A49:F53"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Tipo de producto"/>
-    <tableColumn id="2" name="Largo"/>
-    <tableColumn id="3" name="Ancho"/>
-    <tableColumn id="4" name="Alto"/>
-    <tableColumn id="5" name="Peso/pieza"/>
-    <tableColumn id="6" name="Cant./nivel"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="tblElementosSeguridad_MEZ" displayName="tblElementosSeguridad_MEZ" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="tbl040" displayName="tbl040" ref="A57:G61" headerRowCount="1">
-  <autoFilter ref="A57:G61"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Peso"/>
-    <tableColumn id="2" name="Alto"/>
-    <tableColumn id="3" name="Frente"/>
-    <tableColumn id="4" name="Fondo"/>
-    <tableColumn id="5" name="Huella"/>
-    <tableColumn id="6" name="Exc. frente"/>
-    <tableColumn id="7" name="Exc. fondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="tblPiezasEspeciales_MEZ" displayName="tblPiezasEspeciales_MEZ" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="tbl041" displayName="tbl041" ref="A75:C79" headerRowCount="1">
-  <autoFilter ref="A75:C79"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="tblColores_MEZ" displayName="tblColores_MEZ" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="tbl042" displayName="tbl042" ref="A82:C85" headerRowCount="1">
-  <autoFilter ref="A82:C85"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="tblProveedoresExternos_MEZ" displayName="tblProveedoresExternos_MEZ" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table44.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="tbl043" displayName="tbl043" ref="A94:B98" headerRowCount="1">
-  <autoFilter ref="A94:B98"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="tblPiezas_CFL" displayName="tblPiezas_CFL" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="tbl044" displayName="tbl044" ref="A110:B113" headerRowCount="1">
-  <autoFilter ref="A110:B113"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="tblTarimas_CFL" displayName="tblTarimas_CFL" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="tblProductos_CFL" displayName="tblProductos_CFL" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="tblElementosSeguridad_CFL" displayName="tblElementosSeguridad_CFL" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="tblPiezasEspeciales_CFL" displayName="tblPiezasEspeciales_CFL" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="tblColores_CFL" displayName="tblColores_CFL" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl004" displayName="tbl004" ref="A71:B75" headerRowCount="1">
-  <autoFilter ref="A71:B75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblElementosSeguridad_SEL" displayName="tblElementosSeguridad_SEL" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="tblProveedoresExternos_CFL" displayName="tblProveedoresExternos_CFL" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Color"/>
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table51.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="tblPiezas_MZL" displayName="tblPiezas_MZL" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="tblTarimas_MZL" displayName="tblTarimas_MZL" ref="O4:U29" headerRowCount="1">
+  <autoFilter ref="O4:U29"/>
+  <tableColumns count="7">
+    <tableColumn id="15" name="Peso"/>
+    <tableColumn id="16" name="Alto"/>
+    <tableColumn id="17" name="Frente"/>
+    <tableColumn id="18" name="Fondo"/>
+    <tableColumn id="19" name="Huella"/>
+    <tableColumn id="20" name="ExcedenteFrente"/>
+    <tableColumn id="21" name="ExcedenteFondo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="tblProductos_MZL" displayName="tblProductos_MZL" ref="I32:N57" headerRowCount="1">
+  <autoFilter ref="I32:N57"/>
+  <tableColumns count="6">
+    <tableColumn id="9" name="TipoProducto"/>
+    <tableColumn id="10" name="LargoProducto"/>
+    <tableColumn id="11" name="AnchoProducto"/>
+    <tableColumn id="12" name="AltoProducto"/>
+    <tableColumn id="13" name="PesoProducto"/>
+    <tableColumn id="14" name="CantidadPorNivel"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="tblElementosSeguridad_MZL" displayName="tblElementosSeguridad_MZL" ref="P32:R57" headerRowCount="1">
+  <autoFilter ref="P32:R57"/>
+  <tableColumns count="3">
+    <tableColumn id="16" name="Pieza"/>
+    <tableColumn id="17" name="Cantidad"/>
+    <tableColumn id="18" name="Comentario"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="tblPiezasEspeciales_MZL" displayName="tblPiezasEspeciales_MZL" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="tblColores_MZL" displayName="tblColores_MZL" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="tblProveedoresExternos_MZL" displayName="tblProveedoresExternos_MZL" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tbl005" displayName="tbl005" ref="A87:B90" headerRowCount="1">
-  <autoFilter ref="A87:B90"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Proveedor"/>
-    <tableColumn id="2" name="Alcance"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblPiezasEspeciales_SEL" displayName="tblPiezasEspeciales_SEL" ref="T32:V57" headerRowCount="1">
+  <autoFilter ref="T32:V57"/>
+  <tableColumns count="3">
+    <tableColumn id="20" name="Pieza"/>
+    <tableColumn id="21" name="Cantidad"/>
+    <tableColumn id="22" name="Comentario"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tbl006" displayName="tbl006" ref="A16:E22" headerRowCount="1">
-  <autoFilter ref="A16:E22"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Código"/>
-    <tableColumn id="2" name="Descripción"/>
-    <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Unidad"/>
-    <tableColumn id="5" name="Notas"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblColores_SEL" displayName="tblColores_SEL" ref="I60:J85" headerRowCount="1">
+  <autoFilter ref="I60:J85"/>
+  <tableColumns count="2">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Color"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl007" displayName="tbl007" ref="A60:C64" headerRowCount="1">
-  <autoFilter ref="A60:C64"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblProveedoresExternos_SEL" displayName="tblProveedoresExternos_SEL" ref="L60:M85" headerRowCount="1">
+  <autoFilter ref="L60:M85"/>
+  <tableColumns count="2">
+    <tableColumn id="12" name="Proveedor"/>
+    <tableColumn id="13" name="Alcance"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tbl008" displayName="tbl008" ref="A67:C70" headerRowCount="1">
-  <autoFilter ref="A67:C70"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Pieza"/>
-    <tableColumn id="2" name="Cantidad"/>
-    <tableColumn id="3" name="Comentario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblPiezas_DIN" displayName="tblPiezas_DIN" ref="I4:M29" headerRowCount="1">
+  <autoFilter ref="I4:M29"/>
+  <tableColumns count="5">
+    <tableColumn id="9" name="Pieza"/>
+    <tableColumn id="10" name="Comentarios"/>
+    <tableColumn id="11" name="Cantidad"/>
+    <tableColumn id="12" name="Unidad"/>
+    <tableColumn id="13" name="Notas"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1422,7 +1610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:V115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1619,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1453,6 +1655,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1494,6 +1756,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -1614,6 +1877,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -1696,6 +1960,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1922,6 +2246,7 @@
       <c r="E53" s="10" t="n"/>
       <c r="F53" s="10" t="n"/>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
@@ -1999,6 +2324,26 @@
       <c r="E60" s="10" t="n"/>
       <c r="F60" s="10" t="n"/>
       <c r="G60" s="10" t="n"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -2009,6 +2354,7 @@
       <c r="F61" s="10" t="n"/>
       <c r="G61" s="10" t="n"/>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
@@ -2157,6 +2503,7 @@
       <c r="B79" s="10" t="n"/>
       <c r="C79" s="10" t="n"/>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
         <is>
@@ -2515,6 +2862,34 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FDI Excel layout JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>{"version":1,"configSheet":"FDI_Table_Config","hiddenColumns":["I:V"],"tables":{"piezas":{"baseName":"tblPiezas","range":"I4:M29","headers":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"aliases":[["Pieza","Código","Codigo"],["Comentarios","Comentario","Descripción","Descripcion"],["Cantidad"],["Unidad"],["Notas"]],"previewRanges":{"SEL":"A16:E22","DIN":"A16:E22","PBK":"A16:E22","DRV":"A16:E22","CAN":"A16:E22","MEZ":"A16:E22","CFL":"A16:E22","MZL":"A16:E22"}},"tarimas":{"baseName":"tblTarimas","range":"O4:U29","headers":["Peso","Alto","Frente","Fondo","Huella","ExcedenteFrente","ExcedenteFondo"],"aliases":[["Peso","PesoTarima"],["Alto","AltoTarima"],["Frente","FrenteTarima"],["Fondo","FondoTarima"],["Huella","HuellaTarima"],["ExcedenteFrente","Excedente frente"],["ExcedenteFondo","Excedente fondo"]],"previewRanges":{"MZL":"A57:G61"}},"productos":{"baseName":"tblProductos","range":"I32:N57","headers":["TipoProducto","LargoProducto","AnchoProducto","AltoProducto","PesoProducto","CantidadPorNivel"],"aliases":[["TipoProducto","Tipo producto","Tipo","Producto"],["LargoProducto","Largo"],["AnchoProducto","Ancho"],["AltoProducto","Alto"],["PesoProducto","Peso","PesoPieza"],["CantidadPorNivel","Cantidad por nivel","Cantidad"]],"previewRanges":{"MEZ":"A30:F36","CFL":"A30:F36","MZL":"A49:F53"}},"elementosSeguridad":{"baseName":"tblElementosSeguridad","range":"P32:R57","headers":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza","Elemento"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A52:C56","DIN":"A60:C64","PBK":"A60:C64","DRV":"A62:C66","CAN":"A51:C55","MEZ":"A63:C67","CFL":"A56:C60","MZL":"A75:C79"}},"piezasEspeciales":{"baseName":"tblPiezasEspeciales","range":"T32:V57","headers":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A59:C62","DIN":"A67:C70","PBK":"A67:C70","DRV":"A69:C72","CAN":"A58:C61","MEZ":"A70:C73","CFL":"A63:C66","MZL":"A82:C85"}},"colores":{"baseName":"tblColores","range":"I60:J85","headers":["Pieza","Color"],"aliases":[["Pieza"],["Color","ColorNombre","ColorTexto"]],"previewRanges":{"SEL":"A71:B75","DIN":"A79:B83","PBK":"A79:B83","DRV":"A81:B85","CAN":"A70:B74","MEZ":"A82:B86","CFL":"A75:B79","MZL":"A94:B98"}},"proveedoresExternos":{"baseName":"tblProveedoresExternos","range":"L60:M85","headers":["Proveedor","Alcance"],"aliases":[["Proveedor"],["Alcance","Comentarios"]],"previewRanges":{"SEL":"A87:B90","DIN":"A95:B98","PBK":"A95:B98","DRV":"A97:B100","CAN":"A86:B89","MEZ":"A98:B101","CFL":"A91:B94","MZL":"A110:B113"}}}}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2700,7 +3075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:V92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2709,6 +3084,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2731,6 +3120,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2772,6 +3221,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -2892,6 +3342,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -2974,6 +3425,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -3193,6 +3704,7 @@
       <c r="B56" s="10" t="n"/>
       <c r="C56" s="10" t="n"/>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
@@ -3221,6 +3733,26 @@
       <c r="A60" s="10" t="n"/>
       <c r="B60" s="10" t="n"/>
       <c r="C60" s="10" t="n"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -3232,6 +3764,7 @@
       <c r="B62" s="10" t="n"/>
       <c r="C62" s="10" t="n"/>
     </row>
+    <row r="63"/>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
@@ -3331,6 +3864,7 @@
       <c r="A75" s="10" t="n"/>
       <c r="B75" s="10" t="n"/>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
         <is>
@@ -3526,12 +4060,14 @@
     <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="5">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3542,7 +4078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:V100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3551,6 +4087,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3573,6 +4123,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -3614,6 +4224,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -3734,6 +4345,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -3816,6 +4428,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -4101,6 +4773,26 @@
           <t>Comentario</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -4122,6 +4814,7 @@
       <c r="B64" s="10" t="n"/>
       <c r="C64" s="10" t="n"/>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
@@ -4161,6 +4854,7 @@
       <c r="B70" s="10" t="n"/>
       <c r="C70" s="10" t="n"/>
     </row>
+    <row r="71"/>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
@@ -4260,6 +4954,7 @@
       <c r="A83" s="10" t="n"/>
       <c r="B83" s="10" t="n"/>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
         <is>
@@ -4465,12 +5160,14 @@
     <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="5">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4481,7 +5178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:V100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4490,6 +5187,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4512,6 +5223,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -4553,6 +5324,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -4673,6 +5445,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -4755,6 +5528,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -5040,6 +5873,26 @@
           <t>Comentario</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -5061,6 +5914,7 @@
       <c r="B64" s="10" t="n"/>
       <c r="C64" s="10" t="n"/>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
@@ -5100,6 +5954,7 @@
       <c r="B70" s="10" t="n"/>
       <c r="C70" s="10" t="n"/>
     </row>
+    <row r="71"/>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
@@ -5199,6 +6054,7 @@
       <c r="A83" s="10" t="n"/>
       <c r="B83" s="10" t="n"/>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
         <is>
@@ -5404,12 +6260,14 @@
     <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="5">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5420,7 +6278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:V102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5429,6 +6287,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5451,6 +6323,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -5492,6 +6424,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -5612,6 +6545,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -5694,6 +6628,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -5967,6 +6961,26 @@
       <c r="B60" s="8" t="n"/>
       <c r="C60" s="14" t="n"/>
       <c r="D60" s="15" t="n"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -6012,6 +7026,7 @@
       <c r="B66" s="10" t="n"/>
       <c r="C66" s="10" t="n"/>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
@@ -6051,6 +7066,7 @@
       <c r="B72" s="10" t="n"/>
       <c r="C72" s="10" t="n"/>
     </row>
+    <row r="73"/>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
         <is>
@@ -6356,12 +7372,14 @@
     <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="5">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6372,7 +7390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:V91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6381,6 +7399,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6403,6 +7435,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -6444,6 +7536,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -6564,6 +7657,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -6646,6 +7740,66 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="14" t="n"/>
       <c r="D32" s="15" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -6852,6 +8006,7 @@
       <c r="B55" s="10" t="n"/>
       <c r="C55" s="10" t="n"/>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
@@ -6885,12 +8040,33 @@
       <c r="A60" s="10" t="n"/>
       <c r="B60" s="10" t="n"/>
       <c r="C60" s="10" t="n"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
       <c r="B61" s="10" t="n"/>
       <c r="C61" s="10" t="n"/>
     </row>
+    <row r="62"/>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
@@ -6990,6 +8166,7 @@
       <c r="A74" s="10" t="n"/>
       <c r="B74" s="10" t="n"/>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
@@ -7184,12 +8361,14 @@
     <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="5">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7200,7 +8379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:V103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7209,6 +8388,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7231,6 +8424,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -7272,6 +8525,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -7392,6 +8646,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -7489,6 +8744,66 @@
       <c r="D32" s="10" t="n"/>
       <c r="E32" s="10" t="n"/>
       <c r="F32" s="10" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -7522,6 +8837,7 @@
       <c r="E36" s="10" t="n"/>
       <c r="F36" s="10" t="n"/>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
@@ -7752,6 +9068,26 @@
       <c r="B60" s="8" t="n"/>
       <c r="C60" s="14" t="n"/>
       <c r="D60" s="15" t="n"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -7807,6 +9143,7 @@
       <c r="B67" s="10" t="n"/>
       <c r="C67" s="10" t="n"/>
     </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
@@ -7846,6 +9183,7 @@
       <c r="B73" s="10" t="n"/>
       <c r="C73" s="10" t="n"/>
     </row>
+    <row r="74"/>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
@@ -8145,13 +9483,14 @@
     <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="6">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8162,7 +9501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:V96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8171,6 +9510,20 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -8193,6 +9546,66 @@
           <t>Identificación</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Frente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>ExcedenteFrente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ExcedenteFondo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -8234,6 +9647,7 @@
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -8354,6 +9768,7 @@
       <c r="D22" s="10" t="n"/>
       <c r="E22" s="10" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -8451,6 +9866,66 @@
       <c r="D32" s="10" t="n"/>
       <c r="E32" s="10" t="n"/>
       <c r="F32" s="10" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -8484,6 +9959,7 @@
       <c r="E36" s="10" t="n"/>
       <c r="F36" s="10" t="n"/>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
@@ -8698,7 +10174,28 @@
       <c r="A60" s="10" t="n"/>
       <c r="B60" s="10" t="n"/>
       <c r="C60" s="10" t="n"/>
-    </row>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+    </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
@@ -8738,6 +10235,7 @@
       <c r="B66" s="10" t="n"/>
       <c r="C66" s="10" t="n"/>
     </row>
+    <row r="67"/>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
@@ -8837,6 +10335,7 @@
       <c r="A79" s="10" t="n"/>
       <c r="B79" s="10" t="n"/>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
         <is>
@@ -9030,13 +10529,14 @@
     <mergeCell ref="B86:D86"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="6">
+  <tableParts count="7">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Avoid row inserts around workbook tables
</commit_message>
<xml_diff>
--- a/templates/FDI_Master.xlsx
+++ b/templates/FDI_Master.xlsx
@@ -311,61 +311,61 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblProductos_DIN" displayName="tblProductos_DIN" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblProductos_DIN" displayName="tblProductos_DIN" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblElementosSeguridad_DIN" displayName="tblElementosSeguridad_DIN" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblElementosSeguridad_DIN" displayName="tblElementosSeguridad_DIN" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPiezasEspeciales_DIN" displayName="tblPiezasEspeciales_DIN" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPiezasEspeciales_DIN" displayName="tblPiezasEspeciales_DIN" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblColores_DIN" displayName="tblColores_DIN" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblColores_DIN" displayName="tblColores_DIN" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblProveedoresExternos_DIN" displayName="tblProveedoresExternos_DIN" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblProveedoresExternos_DIN" displayName="tblProveedoresExternos_DIN" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -402,27 +402,27 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblProductos_PBK" displayName="tblProductos_PBK" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblProductos_PBK" displayName="tblProductos_PBK" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblElementosSeguridad_PBK" displayName="tblElementosSeguridad_PBK" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblElementosSeguridad_PBK" displayName="tblElementosSeguridad_PBK" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -443,34 +443,34 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tblPiezasEspeciales_PBK" displayName="tblPiezasEspeciales_PBK" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tblPiezasEspeciales_PBK" displayName="tblPiezasEspeciales_PBK" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tblColores_PBK" displayName="tblColores_PBK" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tblColores_PBK" displayName="tblColores_PBK" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tblProveedoresExternos_PBK" displayName="tblProveedoresExternos_PBK" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="tblProveedoresExternos_PBK" displayName="tblProveedoresExternos_PBK" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -507,61 +507,61 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tblProductos_DRV" displayName="tblProductos_DRV" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="tblProductos_DRV" displayName="tblProductos_DRV" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tblElementosSeguridad_DRV" displayName="tblElementosSeguridad_DRV" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="tblElementosSeguridad_DRV" displayName="tblElementosSeguridad_DRV" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tblPiezasEspeciales_DRV" displayName="tblPiezasEspeciales_DRV" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="tblPiezasEspeciales_DRV" displayName="tblPiezasEspeciales_DRV" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tblColores_DRV" displayName="tblColores_DRV" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="tblColores_DRV" displayName="tblColores_DRV" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tblProveedoresExternos_DRV" displayName="tblProveedoresExternos_DRV" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="tblProveedoresExternos_DRV" displayName="tblProveedoresExternos_DRV" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -614,61 +614,61 @@
 </file>
 
 <file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="tblProductos_CAN" displayName="tblProductos_CAN" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="tblProductos_CAN" displayName="tblProductos_CAN" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="tblElementosSeguridad_CAN" displayName="tblElementosSeguridad_CAN" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="tblElementosSeguridad_CAN" displayName="tblElementosSeguridad_CAN" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="tblPiezasEspeciales_CAN" displayName="tblPiezasEspeciales_CAN" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="tblPiezasEspeciales_CAN" displayName="tblPiezasEspeciales_CAN" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="tblColores_CAN" displayName="tblColores_CAN" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="tblColores_CAN" displayName="tblColores_CAN" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="tblProveedoresExternos_CAN" displayName="tblProveedoresExternos_CAN" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="tblProveedoresExternos_CAN" displayName="tblProveedoresExternos_CAN" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -705,76 +705,76 @@
 </file>
 
 <file path=xl/tables/table39.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="tblProductos_MEZ" displayName="tblProductos_MEZ" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="tblProductos_MEZ" displayName="tblProductos_MEZ" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblProductos_SEL" displayName="tblProductos_SEL" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblProductos_SEL" displayName="tblProductos_SEL" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table40.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="tblElementosSeguridad_MEZ" displayName="tblElementosSeguridad_MEZ" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="tblElementosSeguridad_MEZ" displayName="tblElementosSeguridad_MEZ" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table41.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="tblPiezasEspeciales_MEZ" displayName="tblPiezasEspeciales_MEZ" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="tblPiezasEspeciales_MEZ" displayName="tblPiezasEspeciales_MEZ" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table42.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="tblColores_MEZ" displayName="tblColores_MEZ" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="tblColores_MEZ" displayName="tblColores_MEZ" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table43.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="tblProveedoresExternos_MEZ" displayName="tblProveedoresExternos_MEZ" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="tblProveedoresExternos_MEZ" displayName="tblProveedoresExternos_MEZ" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -811,73 +811,73 @@
 </file>
 
 <file path=xl/tables/table46.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="tblProductos_CFL" displayName="tblProductos_CFL" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="tblProductos_CFL" displayName="tblProductos_CFL" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table47.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="tblElementosSeguridad_CFL" displayName="tblElementosSeguridad_CFL" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="tblElementosSeguridad_CFL" displayName="tblElementosSeguridad_CFL" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table48.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="tblPiezasEspeciales_CFL" displayName="tblPiezasEspeciales_CFL" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="tblPiezasEspeciales_CFL" displayName="tblPiezasEspeciales_CFL" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table49.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="tblColores_CFL" displayName="tblColores_CFL" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="tblColores_CFL" displayName="tblColores_CFL" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblElementosSeguridad_SEL" displayName="tblElementosSeguridad_SEL" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblElementosSeguridad_SEL" displayName="tblElementosSeguridad_SEL" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table50.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="tblProveedoresExternos_CFL" displayName="tblProveedoresExternos_CFL" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="tblProveedoresExternos_CFL" displayName="tblProveedoresExternos_CFL" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -914,95 +914,95 @@
 </file>
 
 <file path=xl/tables/table53.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="tblProductos_MZL" displayName="tblProductos_MZL" ref="I32:N57" headerRowCount="1">
-  <autoFilter ref="I32:N57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="tblProductos_MZL" displayName="tblProductos_MZL" ref="W4:AB29" headerRowCount="1">
+  <autoFilter ref="W4:AB29"/>
   <tableColumns count="6">
-    <tableColumn id="9" name="TipoProducto"/>
-    <tableColumn id="10" name="LargoProducto"/>
-    <tableColumn id="11" name="AnchoProducto"/>
-    <tableColumn id="12" name="AltoProducto"/>
-    <tableColumn id="13" name="PesoProducto"/>
-    <tableColumn id="14" name="CantidadPorNivel"/>
+    <tableColumn id="23" name="TipoProducto"/>
+    <tableColumn id="24" name="LargoProducto"/>
+    <tableColumn id="25" name="AnchoProducto"/>
+    <tableColumn id="26" name="AltoProducto"/>
+    <tableColumn id="27" name="PesoProducto"/>
+    <tableColumn id="28" name="CantidadPorNivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table54.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="tblElementosSeguridad_MZL" displayName="tblElementosSeguridad_MZL" ref="P32:R57" headerRowCount="1">
-  <autoFilter ref="P32:R57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="tblElementosSeguridad_MZL" displayName="tblElementosSeguridad_MZL" ref="AD4:AF29" headerRowCount="1">
+  <autoFilter ref="AD4:AF29"/>
   <tableColumns count="3">
-    <tableColumn id="16" name="Pieza"/>
-    <tableColumn id="17" name="Cantidad"/>
-    <tableColumn id="18" name="Comentario"/>
+    <tableColumn id="30" name="Pieza"/>
+    <tableColumn id="31" name="Cantidad"/>
+    <tableColumn id="32" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table55.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="tblPiezasEspeciales_MZL" displayName="tblPiezasEspeciales_MZL" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="tblPiezasEspeciales_MZL" displayName="tblPiezasEspeciales_MZL" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table56.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="tblColores_MZL" displayName="tblColores_MZL" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="tblColores_MZL" displayName="tblColores_MZL" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table57.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="tblProveedoresExternos_MZL" displayName="tblProveedoresExternos_MZL" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="tblProveedoresExternos_MZL" displayName="tblProveedoresExternos_MZL" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblPiezasEspeciales_SEL" displayName="tblPiezasEspeciales_SEL" ref="T32:V57" headerRowCount="1">
-  <autoFilter ref="T32:V57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblPiezasEspeciales_SEL" displayName="tblPiezasEspeciales_SEL" ref="AH4:AJ29" headerRowCount="1">
+  <autoFilter ref="AH4:AJ29"/>
   <tableColumns count="3">
-    <tableColumn id="20" name="Pieza"/>
-    <tableColumn id="21" name="Cantidad"/>
-    <tableColumn id="22" name="Comentario"/>
+    <tableColumn id="34" name="Pieza"/>
+    <tableColumn id="35" name="Cantidad"/>
+    <tableColumn id="36" name="Comentario"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblColores_SEL" displayName="tblColores_SEL" ref="I60:J85" headerRowCount="1">
-  <autoFilter ref="I60:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblColores_SEL" displayName="tblColores_SEL" ref="AL4:AM29" headerRowCount="1">
+  <autoFilter ref="AL4:AM29"/>
   <tableColumns count="2">
-    <tableColumn id="9" name="Pieza"/>
-    <tableColumn id="10" name="Color"/>
+    <tableColumn id="38" name="Pieza"/>
+    <tableColumn id="39" name="Color"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblProveedoresExternos_SEL" displayName="tblProveedoresExternos_SEL" ref="L60:M85" headerRowCount="1">
-  <autoFilter ref="L60:M85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tblProveedoresExternos_SEL" displayName="tblProveedoresExternos_SEL" ref="AO4:AP29" headerRowCount="1">
+  <autoFilter ref="AO4:AP29"/>
   <tableColumns count="2">
-    <tableColumn id="12" name="Proveedor"/>
-    <tableColumn id="13" name="Alcance"/>
+    <tableColumn id="41" name="Proveedor"/>
+    <tableColumn id="42" name="Alcance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1616,7 +1616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V103"/>
+  <dimension ref="A1:AP103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -1636,6 +1636,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -1716,6 +1736,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2171,6 @@
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
@@ -2377,7 +2476,6 @@
       <c r="B67" s="2" t="n"/>
       <c r="C67" s="2" t="n"/>
     </row>
-    <row r="68"/>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
@@ -2417,7 +2515,6 @@
       <c r="B73" s="2" t="n"/>
       <c r="C73" s="2" t="n"/>
     </row>
-    <row r="74"/>
     <row r="75" ht="20.1" customHeight="1" s="8">
       <c r="A75" s="5" t="inlineStr">
         <is>
@@ -2735,7 +2832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V96"/>
+  <dimension ref="A1:AP96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -2755,6 +2852,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -2835,6 +2952,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3387,6 @@
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
@@ -3426,7 +3622,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
@@ -3466,7 +3661,6 @@
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
     </row>
-    <row r="67"/>
     <row r="68" ht="20.1" customHeight="1" s="8">
       <c r="A68" s="5" t="inlineStr">
         <is>
@@ -3566,7 +3760,6 @@
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="2" t="n"/>
     </row>
-    <row r="80"/>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
         <is>
@@ -3778,7 +3971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V115"/>
+  <dimension ref="A1:AP115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -3798,6 +3991,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -3878,6 +4091,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4704,6 @@
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
@@ -4519,7 +4811,6 @@
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="n"/>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
@@ -4668,7 +4959,6 @@
       <c r="B79" s="2" t="n"/>
       <c r="C79" s="2" t="n"/>
     </row>
-    <row r="80"/>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
         <is>
@@ -5046,7 +5336,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"version":1,"configSheet":"FDI_Table_Config","hiddenColumns":["I:V"],"tables":{"piezas":{"baseName":"tblPiezas","range":"I4:M29","headers":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"previewHeaders":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"aliases":[["Pieza","Código","Codigo"],["Comentarios","Comentario","Descripción","Descripcion"],["Cantidad"],["Unidad"],["Notas"]],"previewRanges":{"SEL":"A16:E22","DIN":"A16:E22","PBK":"A16:E22","DRV":"A16:E22","CAN":"A16:E22","MEZ":"A16:E22","CFL":"A16:E22","MZL":"A16:E22"}},"tarimas":{"baseName":"tblTarimas","range":"O4:U29","headers":["Peso","Alto","Frente","Fondo","Huella","ExcedenteFrente","ExcedenteFondo"],"previewHeaders":["Peso","Alto","Frente","Fondo","Huella","Exc. frente","Exc. fondo"],"aliases":[["Peso","PesoTarima","Pesotarima","Peso tarima"],["Alto","AltoTarima","Altotarima","Alto tarima"],["Frente","FrenteTarima","Frentetarima","Frente tarima"],["Fondo","FondoTarima","Fondotarima","Fondo tarima"],["Huella","HuellaTarima","Huellatarima","Huella tarima"],["ExcedenteFrente","Excedente frente","Excedentefrente"],["ExcedenteFondo","Excedente fondo","Excedentefondo"]],"previewRanges":{"SEL":"A29:G36","DIN":"A29:G36","PBK":"A29:G36","DRV":"A29:G36","MZL":"A57:G61"}},"productos":{"baseName":"tblProductos","range":"I32:N57","headers":["TipoProducto","LargoProducto","AnchoProducto","AltoProducto","PesoProducto","CantidadPorNivel"],"previewHeaders":["Tipo","Largo","Ancho","Alto","Peso","Cant./nivel"],"aliases":[["TipoProducto","Tipo producto","Tipo","Producto"],["LargoProducto","Largo"],["AnchoProducto","Ancho"],["AltoProducto","Alto"],["PesoProducto","Peso","PesoPieza"],["CantidadPorNivel","Cantidad por nivel","Cantidad"]],"previewRanges":{"MEZ":"A30:F36","CFL":"A30:F36","MZL":"A49:F53"}},"elementosSeguridad":{"baseName":"tblElementosSeguridad","range":"P32:R57","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza","Elemento"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A52:C56","DIN":"A60:C64","PBK":"A60:C64","DRV":"A62:C66","CAN":"A51:C55","MEZ":"A63:C67","CFL":"A56:C60","MZL":"A75:C79"}},"piezasEspeciales":{"baseName":"tblPiezasEspeciales","range":"T32:V57","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A59:C62","DIN":"A67:C70","PBK":"A67:C70","DRV":"A69:C72","CAN":"A58:C61","MEZ":"A70:C73","CFL":"A63:C66","MZL":"A82:C85"}},"colores":{"baseName":"tblColores","range":"I60:J85","headers":["Pieza","Color"],"previewHeaders":["Pieza","Color"],"aliases":[["Pieza"],["Color","ColorNombre","ColorTexto"]],"previewRanges":{"SEL":"A71:B75","DIN":"A79:B83","PBK":"A79:B83","DRV":"A81:B85","CAN":"A70:B74","MEZ":"A82:B86","CFL":"A75:B79","MZL":"A94:B98"}},"proveedoresExternos":{"baseName":"tblProveedoresExternos","range":"L60:M85","headers":["Proveedor","Alcance"],"previewHeaders":["Proveedor","Alcance"],"aliases":[["Proveedor"],["Alcance","Comentarios"]],"previewRanges":{"SEL":"A87:B90","DIN":"A95:B98","PBK":"A95:B98","DRV":"A97:B100","CAN":"A86:B89","MEZ":"A98:B101","CFL":"A91:B94","MZL":"A110:B113"}}}}</t>
+          <t>{"version":1,"configSheet":"FDI_Table_Config","hiddenColumns":["I:AP"],"tables":{"piezas":{"baseName":"tblPiezas","range":"I4:M29","headers":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"previewHeaders":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"aliases":[["Pieza","Código","Codigo"],["Comentarios","Comentario","Descripción","Descripcion"],["Cantidad"],["Unidad"],["Notas"]],"previewRanges":{"SEL":"A16:E22","DIN":"A16:E22","PBK":"A16:E22","DRV":"A16:E22","CAN":"A16:E22","MEZ":"A16:E22","CFL":"A16:E22","MZL":"A16:E22"}},"tarimas":{"baseName":"tblTarimas","range":"O4:U29","headers":["Peso","Alto","Frente","Fondo","Huella","ExcedenteFrente","ExcedenteFondo"],"previewHeaders":["Peso","Alto","Frente","Fondo","Huella","Exc. frente","Exc. fondo"],"aliases":[["Peso","PesoTarima","Pesotarima","Peso tarima"],["Alto","AltoTarima","Altotarima","Alto tarima"],["Frente","FrenteTarima","Frentetarima","Frente tarima"],["Fondo","FondoTarima","Fondotarima","Fondo tarima"],["Huella","HuellaTarima","Huellatarima","Huella tarima"],["ExcedenteFrente","Excedente frente","Excedentefrente"],["ExcedenteFondo","Excedente fondo","Excedentefondo"]],"previewRanges":{"SEL":"A29:G36","DIN":"A29:G36","PBK":"A29:G36","DRV":"A29:G36","MZL":"A57:G61"}},"productos":{"baseName":"tblProductos","range":"W4:AB29","headers":["TipoProducto","LargoProducto","AnchoProducto","AltoProducto","PesoProducto","CantidadPorNivel"],"previewHeaders":["Tipo","Largo","Ancho","Alto","Peso","Cant./nivel"],"aliases":[["TipoProducto","Tipo producto","Tipo","Producto"],["LargoProducto","Largo"],["AnchoProducto","Ancho"],["AltoProducto","Alto"],["PesoProducto","Peso","PesoPieza"],["CantidadPorNivel","Cantidad por nivel","Cantidad"]],"previewRanges":{"MEZ":"A30:F36","CFL":"A30:F36","MZL":"A49:F53"}},"elementosSeguridad":{"baseName":"tblElementosSeguridad","range":"AD4:AF29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza","Elemento"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A52:C56","DIN":"A60:C64","PBK":"A60:C64","DRV":"A62:C66","CAN":"A51:C55","MEZ":"A63:C67","CFL":"A56:C60","MZL":"A75:C79"}},"piezasEspeciales":{"baseName":"tblPiezasEspeciales","range":"AH4:AJ29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A59:C62","DIN":"A67:C70","PBK":"A67:C70","DRV":"A69:C72","CAN":"A58:C61","MEZ":"A70:C73","CFL":"A63:C66","MZL":"A82:C85"}},"colores":{"baseName":"tblColores","range":"AL4:AM29","headers":["Pieza","Color"],"previewHeaders":["Pieza","Color"],"aliases":[["Pieza"],["Color","ColorNombre","ColorTexto"]],"previewRanges":{"SEL":"A71:B75","DIN":"A79:B83","PBK":"A79:B83","DRV":"A81:B85","CAN":"A70:B74","MEZ":"A82:B86","CFL":"A75:B79","MZL":"A94:B98"}},"proveedoresExternos":{"baseName":"tblProveedoresExternos","range":"AO4:AP29","headers":["Proveedor","Alcance"],"previewHeaders":["Proveedor","Alcance"],"aliases":[["Proveedor"],["Alcance","Comentarios"]],"previewRanges":{"SEL":"A87:B90","DIN":"A95:B98","PBK":"A95:B98","DRV":"A97:B100","CAN":"A86:B89","MEZ":"A98:B101","CFL":"A91:B94","MZL":"A110:B113"}}}}</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V92"/>
+  <dimension ref="A1:AP92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -6270,6 +6560,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -6350,6 +6660,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -6861,7 +7251,6 @@
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
@@ -6921,7 +7310,6 @@
       <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="n"/>
     </row>
-    <row r="63"/>
     <row r="64" ht="20.1" customHeight="1" s="8">
       <c r="A64" s="5" t="inlineStr">
         <is>
@@ -7021,7 +7409,6 @@
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="2" t="n"/>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
@@ -7227,7 +7614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V100"/>
+  <dimension ref="A1:AP100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -7247,6 +7634,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -7327,6 +7734,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -7945,7 +8432,6 @@
       <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="n"/>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
@@ -7985,7 +8471,6 @@
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="n"/>
     </row>
-    <row r="71"/>
     <row r="72" ht="20.1" customHeight="1" s="8">
       <c r="A72" s="5" t="inlineStr">
         <is>
@@ -8085,7 +8570,6 @@
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="2" t="n"/>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
@@ -8301,7 +8785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V100"/>
+  <dimension ref="A1:AP100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -8321,6 +8805,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -8401,6 +8905,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -9019,7 +9603,6 @@
       <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="n"/>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
@@ -9059,7 +9642,6 @@
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="n"/>
     </row>
-    <row r="71"/>
     <row r="72" ht="20.1" customHeight="1" s="8">
       <c r="A72" s="5" t="inlineStr">
         <is>
@@ -9159,7 +9741,6 @@
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="2" t="n"/>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
@@ -9375,7 +9956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V102"/>
+  <dimension ref="A1:AP102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -9395,6 +9976,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -9475,6 +10076,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -10105,7 +10786,6 @@
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="n"/>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
@@ -10145,7 +10825,6 @@
       <c r="B72" s="2" t="n"/>
       <c r="C72" s="2" t="n"/>
     </row>
-    <row r="73"/>
     <row r="74" ht="20.1" customHeight="1" s="8">
       <c r="A74" s="5" t="inlineStr">
         <is>
@@ -10461,7 +11140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V91"/>
+  <dimension ref="A1:AP91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" style="8" min="1" max="1"/>
@@ -10481,6 +11160,26 @@
     <col hidden="1" width="13" customWidth="1" style="8" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" style="8" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="41" max="41"/>
+    <col hidden="1" width="13" customWidth="1" style="8" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="8">
@@ -10561,6 +11260,86 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>TipoProducto</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LargoProducto</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AnchoProducto</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>AltoProducto</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>PesoProducto</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>CantidadPorNivel</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Pieza</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
         </is>
       </c>
     </row>
@@ -11074,7 +11853,6 @@
       <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="n"/>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
@@ -11134,7 +11912,6 @@
       <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="n"/>
     </row>
-    <row r="62"/>
     <row r="63" ht="20.1" customHeight="1" s="8">
       <c r="A63" s="5" t="inlineStr">
         <is>
@@ -11234,7 +12011,6 @@
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="2" t="n"/>
     </row>
-    <row r="75"/>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(fdi-excel): tabla de tarimas con columnas reales (Tipo/Excedente, sin Huella)
La tabla de tarimas estaba definida con Peso/Alto/Frente/Fondo/Huella/Exc, que
no coincidía con lo capturado por la app (Hija Tarima): el Tipo se perdía y
Peso/Huella salían vacíos. Ahora son 8 columnas:
Tipo | Peso | Alto | Frente | Fondo | Excedente | ExcedenteFrente | ExcedenteFondo
(Huella sale de la tabla: es campo aparte por sistema).

- fdi-excel-layout.json: tarimas 8 cols, range O4:V29, previewRanges A29:H36/A57:H61
- fill-fdi-workbook.ts (Office Script) + generate-fdi-excel.py: TARIMAS_ALIASES/RANGES espejo
- FDI_Master.xlsx: regenerado con --normalize-template (tblTarimas O4:V29 + config sheet)
- payload de muestra: SEL tarima con Peso/Excedente

Verificado corriendo el generador: SEL renderiza las 8 columnas con datos; el
resto de tablas (elementos seguridad, piezas especiales) intactas.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/FDI_Master.xlsx
+++ b/templates/FDI_Master.xlsx
@@ -295,16 +295,17 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblTarimas_DIN" displayName="tblTarimas_DIN" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblTarimas_DIN" displayName="tblTarimas_DIN" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -386,16 +387,17 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblTarimas_PBK" displayName="tblTarimas_PBK" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblTarimas_PBK" displayName="tblTarimas_PBK" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -491,16 +493,17 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tblTarimas_DRV" displayName="tblTarimas_DRV" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="tblTarimas_DRV" displayName="tblTarimas_DRV" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -568,16 +571,17 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblTarimas_SEL" displayName="tblTarimas_SEL" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblTarimas_SEL" displayName="tblTarimas_SEL" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -598,16 +602,17 @@
 </file>
 
 <file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tblTarimas_CAN" displayName="tblTarimas_CAN" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="tblTarimas_CAN" displayName="tblTarimas_CAN" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -689,16 +694,17 @@
 </file>
 
 <file path=xl/tables/table38.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="tblTarimas_MEZ" displayName="tblTarimas_MEZ" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="tblTarimas_MEZ" displayName="tblTarimas_MEZ" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -795,16 +801,17 @@
 </file>
 
 <file path=xl/tables/table45.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="tblTarimas_CFL" displayName="tblTarimas_CFL" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="tblTarimas_CFL" displayName="tblTarimas_CFL" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -898,16 +905,17 @@
 </file>
 
 <file path=xl/tables/table52.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="tblTarimas_MZL" displayName="tblTarimas_MZL" ref="O4:U29" headerRowCount="1">
-  <autoFilter ref="O4:U29"/>
-  <tableColumns count="7">
-    <tableColumn id="15" name="Peso"/>
-    <tableColumn id="16" name="Alto"/>
-    <tableColumn id="17" name="Frente"/>
-    <tableColumn id="18" name="Fondo"/>
-    <tableColumn id="19" name="Huella"/>
-    <tableColumn id="20" name="ExcedenteFrente"/>
-    <tableColumn id="21" name="ExcedenteFondo"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="tblTarimas_MZL" displayName="tblTarimas_MZL" ref="O4:V29" headerRowCount="1">
+  <autoFilter ref="O4:V29"/>
+  <tableColumns count="8">
+    <tableColumn id="15" name="Tipo"/>
+    <tableColumn id="16" name="Peso"/>
+    <tableColumn id="17" name="Alto"/>
+    <tableColumn id="18" name="Frente"/>
+    <tableColumn id="19" name="Fondo"/>
+    <tableColumn id="20" name="Excedente"/>
+    <tableColumn id="21" name="ExcedenteFrente"/>
+    <tableColumn id="22" name="ExcedenteFondo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1705,35 +1713,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -2921,35 +2934,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -4060,35 +4078,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -4721,37 +4744,42 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Exc. frente</t>
+          <t>Excedente</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Exc. fondo</t>
+          <t>Frente exced.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Fondo exced.</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5364,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"version":1,"configSheet":"FDI_Table_Config","hiddenColumns":["I:AP"],"tables":{"piezas":{"baseName":"tblPiezas","range":"I4:M29","headers":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"previewHeaders":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"aliases":[["Pieza","Código","Codigo"],["Comentarios","Comentario","Descripción","Descripcion"],["Cantidad"],["Unidad"],["Notas"]],"previewRanges":{"SEL":"A16:E22","DIN":"A16:E22","PBK":"A16:E22","DRV":"A16:E22","CAN":"A16:E22","MEZ":"A16:E22","CFL":"A16:E22","MZL":"A16:E22"}},"tarimas":{"baseName":"tblTarimas","range":"O4:U29","headers":["Peso","Alto","Frente","Fondo","Huella","ExcedenteFrente","ExcedenteFondo"],"previewHeaders":["Peso","Alto","Frente","Fondo","Huella","Exc. frente","Exc. fondo"],"aliases":[["Peso","PesoTarima","Pesotarima","Peso tarima"],["Alto","AltoTarima","Altotarima","Alto tarima"],["Frente","FrenteTarima","Frentetarima","Frente tarima"],["Fondo","FondoTarima","Fondotarima","Fondo tarima"],["Huella","HuellaTarima","Huellatarima","Huella tarima"],["ExcedenteFrente","Excedente frente","Excedentefrente"],["ExcedenteFondo","Excedente fondo","Excedentefondo"]],"previewRanges":{"SEL":"A29:G36","DIN":"A29:G36","PBK":"A29:G36","DRV":"A29:G36","MZL":"A57:G61"}},"productos":{"baseName":"tblProductos","range":"W4:AB29","headers":["TipoProducto","LargoProducto","AnchoProducto","AltoProducto","PesoProducto","CantidadPorNivel"],"previewHeaders":["Tipo","Largo","Ancho","Alto","Peso","Cant./nivel"],"aliases":[["TipoProducto","Tipo producto","Tipo","Producto"],["LargoProducto","Largo"],["AnchoProducto","Ancho"],["AltoProducto","Alto"],["PesoProducto","Peso","PesoPieza"],["CantidadPorNivel","Cantidad por nivel","Cantidad"]],"previewRanges":{"MEZ":"A30:F36","CFL":"A30:F36","MZL":"A49:F53"}},"elementosSeguridad":{"baseName":"tblElementosSeguridad","range":"AD4:AF29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza","Elemento"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A52:C56","DIN":"A60:C64","PBK":"A60:C64","DRV":"A62:C66","CAN":"A51:C55","MEZ":"A63:C67","CFL":"A56:C60","MZL":"A75:C79"}},"piezasEspeciales":{"baseName":"tblPiezasEspeciales","range":"AH4:AJ29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A59:C62","DIN":"A67:C70","PBK":"A67:C70","DRV":"A69:C72","CAN":"A58:C61","MEZ":"A70:C73","CFL":"A63:C66","MZL":"A82:C85"}},"colores":{"baseName":"tblColores","range":"AL4:AM29","headers":["Pieza","Color"],"previewHeaders":["Pieza","Color"],"aliases":[["Pieza"],["Color","ColorNombre","ColorTexto"]],"previewRanges":{"SEL":"A71:B75","DIN":"A79:B83","PBK":"A79:B83","DRV":"A81:B85","CAN":"A70:B74","MEZ":"A82:B86","CFL":"A75:B79","MZL":"A94:B98"}},"proveedoresExternos":{"baseName":"tblProveedoresExternos","range":"AO4:AP29","headers":["Proveedor","Alcance"],"previewHeaders":["Proveedor","Alcance"],"aliases":[["Proveedor"],["Alcance","Comentarios"]],"previewRanges":{"SEL":"A87:B90","DIN":"A95:B98","PBK":"A95:B98","DRV":"A97:B100","CAN":"A86:B89","MEZ":"A98:B101","CFL":"A91:B94","MZL":"A110:B113"}}}}</t>
+          <t>{"version":1,"configSheet":"FDI_Table_Config","hiddenColumns":["I:AP"],"tables":{"piezas":{"baseName":"tblPiezas","range":"I4:M29","headers":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"previewHeaders":["Pieza","Comentarios","Cantidad","Unidad","Notas"],"aliases":[["Pieza","Código","Codigo"],["Comentarios","Comentario","Descripción","Descripcion"],["Cantidad"],["Unidad"],["Notas"]],"previewRanges":{"SEL":"A16:E22","DIN":"A16:E22","PBK":"A16:E22","DRV":"A16:E22","CAN":"A16:E22","MEZ":"A16:E22","CFL":"A16:E22","MZL":"A16:E22"}},"tarimas":{"baseName":"tblTarimas","range":"O4:V29","headers":["Tipo","Peso","Alto","Frente","Fondo","Excedente","ExcedenteFrente","ExcedenteFondo"],"previewHeaders":["Tipo","Peso","Alto","Frente","Fondo","Excedente","Frente exced.","Fondo exced."],"aliases":[["Tipo","TipoTarima","Tipotarima","Tipo tarima"],["Peso","PesoTarima","Pesotarima","Peso tarima"],["Alto","AltoTarima","Altotarima","Alto tarima"],["Frente","FrenteTarima","Frentetarima","Frente tarima"],["Fondo","FondoTarima","Fondotarima","Fondo tarima"],["Excedente","¿Excedente?","ExcedenteTarima","Excedente?","Excedente tarima"],["ExcedenteFrente","Excedente frente","Excedentefrente","FrenteExcedente"],["ExcedenteFondo","Excedente fondo","Excedentefondo","FondoExcedente"]],"previewRanges":{"SEL":"A29:H36","DIN":"A29:H36","PBK":"A29:H36","DRV":"A29:H36","MZL":"A57:H61"}},"productos":{"baseName":"tblProductos","range":"W4:AB29","headers":["TipoProducto","LargoProducto","AnchoProducto","AltoProducto","PesoProducto","CantidadPorNivel"],"previewHeaders":["Tipo","Largo","Ancho","Alto","Peso","Cant./nivel"],"aliases":[["TipoProducto","Tipo producto","Tipo","Producto"],["LargoProducto","Largo"],["AnchoProducto","Ancho"],["AltoProducto","Alto"],["PesoProducto","Peso","PesoPieza"],["CantidadPorNivel","Cantidad por nivel","Cantidad"]],"previewRanges":{"MEZ":"A30:F36","CFL":"A30:F36","MZL":"A49:F53"}},"elementosSeguridad":{"baseName":"tblElementosSeguridad","range":"AD4:AF29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza","Elemento"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A52:C56","DIN":"A60:C64","PBK":"A60:C64","DRV":"A62:C66","CAN":"A51:C55","MEZ":"A63:C67","CFL":"A56:C60","MZL":"A75:C79"}},"piezasEspeciales":{"baseName":"tblPiezasEspeciales","range":"AH4:AJ29","headers":["Pieza","Cantidad","Comentario"],"previewHeaders":["Pieza","Cantidad","Comentario"],"aliases":[["Pieza"],["Cantidad"],["Comentario","Comentarios"]],"previewRanges":{"SEL":"A59:C62","DIN":"A67:C70","PBK":"A67:C70","DRV":"A69:C72","CAN":"A58:C61","MEZ":"A70:C73","CFL":"A63:C66","MZL":"A82:C85"}},"colores":{"baseName":"tblColores","range":"AL4:AM29","headers":["Pieza","Color"],"previewHeaders":["Pieza","Color"],"aliases":[["Pieza"],["Color","ColorNombre","ColorTexto"]],"previewRanges":{"SEL":"A71:B75","DIN":"A79:B83","PBK":"A79:B83","DRV":"A81:B85","CAN":"A70:B74","MEZ":"A82:B86","CFL":"A75:B79","MZL":"A94:B98"}},"proveedoresExternos":{"baseName":"tblProveedoresExternos","range":"AO4:AP29","headers":["Proveedor","Alcance"],"previewHeaders":["Proveedor","Alcance"],"aliases":[["Proveedor"],["Alcance","Comentarios"]],"previewRanges":{"SEL":"A87:B90","DIN":"A95:B98","PBK":"A95:B98","DRV":"A97:B100","CAN":"A86:B89","MEZ":"A98:B101","CFL":"A91:B94","MZL":"A110:B113"}}}}</t>
         </is>
       </c>
     </row>
@@ -6629,35 +6657,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -6951,37 +6984,42 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Exc. frente</t>
+          <t>Excedente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Exc. fondo</t>
+          <t>Frente exced.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fondo exced.</t>
         </is>
       </c>
     </row>
@@ -7703,35 +7741,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -8025,37 +8068,42 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Exc. frente</t>
+          <t>Excedente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Exc. fondo</t>
+          <t>Frente exced.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fondo exced.</t>
         </is>
       </c>
     </row>
@@ -8874,35 +8922,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -9196,37 +9249,42 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Exc. frente</t>
+          <t>Excedente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Exc. fondo</t>
+          <t>Frente exced.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fondo exced.</t>
         </is>
       </c>
     </row>
@@ -10045,35 +10103,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>
@@ -10367,37 +10430,42 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Exc. frente</t>
+          <t>Excedente</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Exc. fondo</t>
+          <t>Frente exced.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fondo exced.</t>
         </is>
       </c>
     </row>
@@ -11229,35 +11297,40 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Frente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Huella</t>
-        </is>
-      </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>Excedente</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>ExcedenteFrente</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>ExcedenteFondo</t>
         </is>

</xml_diff>